<commit_message>
chore: 발송 이력·누적 기록 갱신 2026-09-14T06:17Z
</commit_message>
<xml_diff>
--- a/공고누적.xlsx
+++ b/공고누적.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공고누적" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -494,32 +494,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>한국사회적기업진흥원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
+          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -531,32 +531,32 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>전남정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -568,32 +568,32 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>한국산업기술진흥원(KIAT)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>표창</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -605,28 +605,32 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>고령친화산업지원센터</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -638,28 +642,32 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>고령친화산업지원센터</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -671,32 +679,32 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -708,27 +716,27 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국사회적기업진흥원</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
+          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -745,22 +753,22 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -770,7 +778,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -782,32 +790,32 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>수출, 스마트</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -819,32 +827,28 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -856,32 +860,28 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -898,17 +898,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
+          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -935,27 +935,27 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
+          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -972,27 +972,27 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
+          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1009,27 +1009,27 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
+          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>수출, 스마트</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1046,27 +1046,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1083,27 +1083,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>마케팅, 홍보</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1120,27 +1120,27 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1157,27 +1157,27 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1194,27 +1194,27 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1231,27 +1231,27 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1268,27 +1268,27 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, AX</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1305,27 +1305,27 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>마케팅, 홍보</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1342,27 +1342,27 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1394,12 +1394,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1416,27 +1416,27 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>산업통상부</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1453,23 +1453,27 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>광주정보문화산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr"/>
+          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1486,23 +1490,27 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr"/>
+          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>에이지테크, AX</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1519,33 +1527,247 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
+          <t>부산정보산업진흥원</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>에이지테크, 실증</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>광주테크노파크</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>실증</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>광주테크노파크</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Age-Tech</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>산업통상부</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>광주정보문화산업진흥원</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
           <t>고령친화산업지원센터</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>고령</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>고령, 유공, 포상</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="G36" s="4" t="inlineStr">
         <is>
           <t>바로가기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G30"/>
+  <autoFilter ref="A1:G36"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -1576,6 +1798,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId35"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: 발송 이력·누적 기록 갱신 2026-09-14T14:41Z
</commit_message>
<xml_diff>
--- a/공고누적.xlsx
+++ b/공고누적.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공고누적" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -499,12 +499,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>한국산업기술진흥원(KIAT)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
+          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -514,12 +514,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>표창</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -573,12 +573,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>한국산업기술진흥원(KIAT)</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
+          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -588,12 +588,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>표창</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -610,27 +610,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -647,27 +647,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -684,27 +684,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -716,32 +716,32 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>한국사회적기업진흥원</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -753,7 +753,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -790,7 +790,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -832,15 +832,19 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국사회적기업진흥원</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
+          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -848,7 +852,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -865,23 +869,27 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -893,32 +901,32 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -930,32 +938,28 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -967,32 +971,28 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1009,17 +1009,17 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
+          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>수출, 스마트</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1046,27 +1046,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1083,27 +1083,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
+          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1125,12 +1125,12 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
+          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>수출, 스마트</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1157,27 +1157,27 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1194,27 +1194,27 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
+          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1231,27 +1231,27 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
+          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1273,22 +1273,22 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1305,27 +1305,27 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>마케팅, 홍보</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1342,27 +1342,27 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1379,27 +1379,27 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1416,27 +1416,27 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>마케팅, 홍보</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1453,22 +1453,22 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1490,12 +1490,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1505,12 +1505,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, AX</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1527,12 +1527,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1542,12 +1542,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1564,12 +1564,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1579,12 +1579,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1601,12 +1601,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>에이지테크, AX</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1638,27 +1638,27 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>산업통상부</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>에이지테크, 실증</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1675,23 +1675,27 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>광주정보문화산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr"/>
+          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1708,23 +1712,27 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr"/>
+          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1741,33 +1749,136 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
+          <t>산업통상부</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>광주정보문화산업진흥원</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
           <t>고령친화산업지원센터</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>고령</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>고령, 유공, 포상</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="G39" s="4" t="inlineStr">
         <is>
           <t>바로가기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G36"/>
+  <autoFilter ref="A1:G39"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -1804,6 +1915,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: 발송 이력·누적 기록 갱신 2026-09-16T05:47Z
</commit_message>
<xml_diff>
--- a/공고누적.xlsx
+++ b/공고누적.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공고누적" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -494,32 +494,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>한국산업기술진흥원(KIAT)</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
+          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>표창</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -531,32 +531,32 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>전남정보문화산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
+          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -568,32 +568,32 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
+          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -605,22 +605,22 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
+          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -642,32 +642,32 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
+          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -679,32 +679,32 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -721,27 +721,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>한국산업기술진흥원(KIAT)</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>표창</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -758,27 +758,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -795,27 +795,27 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -827,32 +827,32 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>한국사회적기업진흥원</t>
+          <t>전남정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
+          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -864,32 +864,32 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -901,32 +901,32 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -938,28 +938,32 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>고령친화산업지원센터</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -971,28 +975,32 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>고령친화산업지원센터</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1004,32 +1012,32 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1041,27 +1049,27 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국사회적기업진흥원</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
+          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1078,22 +1086,22 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1103,7 +1111,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1115,32 +1123,32 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>수출, 스마트</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1152,32 +1160,28 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1189,32 +1193,28 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1231,17 +1231,17 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
+          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1268,27 +1268,27 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
+          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1305,27 +1305,27 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
+          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1342,27 +1342,27 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
+          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>수출, 스마트</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1379,27 +1379,27 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1416,27 +1416,27 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>마케팅, 홍보</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1453,27 +1453,27 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1490,27 +1490,27 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1527,27 +1527,27 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1564,27 +1564,27 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1601,27 +1601,27 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, AX</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1638,27 +1638,27 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>마케팅, 홍보</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1675,27 +1675,27 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1712,12 +1712,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1727,12 +1727,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1749,27 +1749,27 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>산업통상부</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1786,23 +1786,27 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>광주정보문화산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr"/>
+          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1819,23 +1823,27 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr"/>
+          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>에이지테크, AX</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -1852,33 +1860,247 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
+          <t>부산정보산업진흥원</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>에이지테크, 실증</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>광주테크노파크</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>실증</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>광주테크노파크</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Age-Tech</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>산업통상부</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>광주정보문화산업진흥원</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
           <t>고령친화산업지원센터</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>고령</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr"/>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>고령, 유공, 포상</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr">
+      <c r="G45" s="4" t="inlineStr">
         <is>
           <t>바로가기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G39"/>
+  <autoFilter ref="A1:G45"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -1918,6 +2140,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: 발송 이력·누적 기록 갱신 2026-09-18T05:42Z
</commit_message>
<xml_diff>
--- a/공고누적.xlsx
+++ b/공고누적.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공고누적" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -494,32 +494,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
+          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -531,32 +531,28 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -568,32 +564,28 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -605,32 +597,28 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -642,32 +630,32 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -679,32 +667,32 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
+          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -716,32 +704,32 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>K-Startup(창업진흥원)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>한국산업기술진흥원(KIAT)</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>표창</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -753,32 +741,32 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -790,32 +778,32 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -827,32 +815,32 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>전남정보문화산업진흥원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -864,22 +852,22 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
+          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -889,7 +877,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -901,27 +889,27 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
+          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -938,32 +926,32 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -975,32 +963,32 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1012,32 +1000,32 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1049,32 +1037,32 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>K-Startup(창업진흥원)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>한국사회적기업진흥원</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1086,32 +1074,32 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>한국산업기술진흥원(KIAT)</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>표창</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1123,32 +1111,32 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1160,28 +1148,32 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
+          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1193,28 +1185,32 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>전남정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
+          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1226,32 +1222,32 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
+          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1263,32 +1259,32 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
+          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1300,32 +1296,32 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1337,32 +1333,32 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>수출, 스마트</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1374,7 +1370,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1411,32 +1407,32 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>한국사회적기업진흥원</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
+          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1448,32 +1444,32 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1485,32 +1481,32 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1522,32 +1518,28 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1559,32 +1551,28 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1601,27 +1589,27 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1638,27 +1626,27 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>마케팅, 홍보</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1675,27 +1663,27 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1712,27 +1700,27 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>수출, 스마트</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1749,27 +1737,27 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1786,27 +1774,27 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1823,27 +1811,27 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, AX</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -1860,27 +1848,27 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -1897,27 +1885,27 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -1934,27 +1922,27 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -1971,27 +1959,27 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>산업통상부</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -2008,23 +1996,27 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>광주정보문화산업진흥원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr"/>
+          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>마케팅, 홍보</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2041,23 +2033,27 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr"/>
+          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -2074,33 +2070,395 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
+          <t>중앙사회서비스원</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>사회서비스</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>중소벤처기업부</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>중소벤처기업부</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>유공, 포상</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>부산정보산업진흥원</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>에이지테크, AX</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>부산정보산업진흥원</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>에이지테크, 실증</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>광주테크노파크</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>실증</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>광주테크노파크</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Age-Tech</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>산업통상부</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>광주정보문화산업진흥원</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr"/>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
           <t>고령친화산업지원센터</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr"/>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>고령</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
         <is>
           <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr"/>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr"/>
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>고령, 유공, 포상</t>
         </is>
       </c>
-      <c r="G45" s="4" t="inlineStr">
+      <c r="G55" s="4" t="inlineStr">
         <is>
           <t>바로가기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G45"/>
+  <autoFilter ref="A1:G55"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -2146,6 +2504,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId54"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: 발송 이력·누적 기록 갱신 2026-09-21T00:13Z
</commit_message>
<xml_diff>
--- a/공고누적.xlsx
+++ b/공고누적.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공고누적" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -494,32 +494,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -536,23 +536,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2026 고령친화산업 성과교류회 개최 안내</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
+          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -574,7 +578,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -607,7 +611,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
@@ -618,7 +622,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -630,32 +634,28 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -672,12 +672,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -709,27 +709,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
+          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -746,27 +746,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -798,12 +798,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -825,22 +825,22 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -852,22 +852,22 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
+          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
+          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -946,12 +946,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -963,32 +963,32 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1005,12 +1005,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
+          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1042,27 +1042,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
+          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1074,32 +1074,32 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>한국산업기술진흥원(KIAT)</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
+          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>표창</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1116,12 +1116,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>한국산업기술진흥원(KIAT)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1131,12 +1131,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>표창</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1153,12 +1153,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1168,12 +1168,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1190,12 +1190,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>전남정보문화산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
+          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1205,12 +1205,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1227,12 +1227,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>전남정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
+          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1242,12 +1242,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1264,12 +1264,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
+          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1279,12 +1279,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1301,27 +1301,27 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1353,12 +1353,12 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1380,22 +1380,22 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1407,32 +1407,32 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>한국사회적기업진흥원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1449,12 +1449,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>한국사회적기업진흥원</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1464,12 +1464,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1491,22 +1491,22 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1523,23 +1523,27 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1561,7 +1565,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr"/>
@@ -1572,7 +1576,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1584,24 +1588,20 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1626,27 +1626,27 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
+          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1663,12 +1663,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
+          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1678,12 +1678,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1700,12 +1700,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
+          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1715,12 +1715,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>수출, 스마트</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1737,27 +1737,27 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>수출, 스마트</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1774,12 +1774,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1789,12 +1789,12 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1811,12 +1811,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
+          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1826,12 +1826,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -1848,22 +1848,22 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
+          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1885,12 +1885,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
+          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1900,12 +1900,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -1922,12 +1922,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
+          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1937,12 +1937,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -1959,27 +1959,27 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -1996,27 +1996,27 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>마케팅, 홍보</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2033,27 +2033,27 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>마케팅, 홍보</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -2070,27 +2070,27 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -2107,12 +2107,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2122,12 +2122,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -2181,12 +2181,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2196,12 +2196,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, AX</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>에이지테크, AX</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -2255,12 +2255,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -2270,12 +2270,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>에이지테크, 실증</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2307,12 +2307,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -2329,27 +2329,27 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>산업통상부</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -2366,18 +2366,22 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>광주정보문화산업진흥원</t>
+          <t>산업통상부</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr"/>
+          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2399,23 +2403,23 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>광주정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr"/>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -2437,7 +2441,7 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr"/>
@@ -2448,17 +2452,50 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
+          <t>고령</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
           <t>고령, 유공, 포상</t>
         </is>
       </c>
-      <c r="G55" s="4" t="inlineStr">
+      <c r="G56" s="4" t="inlineStr">
         <is>
           <t>바로가기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G55"/>
+  <autoFilter ref="A1:G56"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -2514,6 +2551,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: 발송 이력·누적 기록 갱신 2026-09-21T03:52Z
</commit_message>
<xml_diff>
--- a/공고누적.xlsx
+++ b/공고누적.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공고누적" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -499,27 +499,27 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>2026년 성능인증(EPC) 신규신청 접수 공고(제4차)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -531,32 +531,32 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
+          <t>구로구 청년창업지원센터 일반 창업교육(하반기: 4회차): 온라인 마케팅 실전 가이드</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>마케팅</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -568,28 +568,32 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026 고령친화산업 성과교류회 개최 안내</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -606,23 +610,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
+          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -644,7 +652,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
@@ -655,7 +663,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -667,32 +675,28 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -704,32 +708,28 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -746,27 +746,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -783,27 +783,27 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -820,27 +820,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -862,22 +862,22 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -889,32 +889,32 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -926,32 +926,32 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
+          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -983,12 +983,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1000,32 +1000,32 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1037,32 +1037,32 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
+          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1079,27 +1079,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
+          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1111,32 +1111,32 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>한국산업기술진흥원(KIAT)</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
+          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>표창</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1148,32 +1148,32 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1190,12 +1190,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국산업기술진흥원(KIAT)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
+          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1205,12 +1205,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>표창</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1227,12 +1227,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>전남정보문화산업진흥원</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1242,12 +1242,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1264,12 +1264,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
+          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1279,12 +1279,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1301,12 +1301,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>전남정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
+          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1316,12 +1316,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1338,27 +1338,27 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1375,17 +1375,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1417,22 +1417,22 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1444,32 +1444,32 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>한국사회적기업진흥원</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1481,7 +1481,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1491,22 +1491,22 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1523,27 +1523,27 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>한국사회적기업진흥원</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1560,23 +1560,27 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr"/>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1593,23 +1597,27 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr"/>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1621,24 +1629,20 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -1646,7 +1650,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1658,32 +1662,28 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1700,27 +1700,27 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
+          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1737,12 +1737,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
+          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1752,12 +1752,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>수출, 스마트</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1774,27 +1774,27 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1811,27 +1811,27 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
+          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>수출, 스마트</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -1848,12 +1848,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1863,12 +1863,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -1885,27 +1885,27 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
+          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -1922,27 +1922,27 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
+          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
+          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1974,12 +1974,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -1996,27 +1996,27 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2033,27 +2033,27 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>마케팅, 홍보</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -2070,27 +2070,27 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -2107,27 +2107,27 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>마케팅, 홍보</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -2144,27 +2144,27 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -2181,12 +2181,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2196,12 +2196,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -2218,12 +2218,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -2233,12 +2233,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, AX</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -2255,12 +2255,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -2270,12 +2270,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -2292,12 +2292,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2307,12 +2307,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>에이지테크, AX</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -2329,12 +2329,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>에이지테크, 실증</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -2366,27 +2366,27 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>산업통상부</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -2403,23 +2403,27 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>광주정보문화산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr"/>
+          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -2436,15 +2440,19 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>산업통상부</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr"/>
+          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -2452,7 +2460,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -2469,33 +2477,99 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>광주정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr"/>
       <c r="E56" s="2" t="inlineStr">
         <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
           <t>확인필요</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>고령</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>고령, 유공, 포상</t>
         </is>
       </c>
-      <c r="G56" s="4" t="inlineStr">
+      <c r="G58" s="4" t="inlineStr">
         <is>
           <t>바로가기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G56"/>
+  <autoFilter ref="A1:G58"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -2552,6 +2626,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: 발송 이력·누적 기록 갱신 2026-09-23T03:49Z
</commit_message>
<xml_diff>
--- a/공고누적.xlsx
+++ b/공고누적.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공고누적" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -494,32 +494,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2026년 성능인증(EPC) 신규신청 접수 공고(제4차)</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -531,32 +531,32 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>구로구 청년창업지원센터 일반 창업교육(하반기: 4회차): 온라인 마케팅 실전 가이드</t>
+          <t>[부산환경운동연합] 원자력안전위원회 최원호 위원장 사퇴 촉구 기자회견</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>마케팅</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -568,32 +568,32 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 계획 공고</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -605,32 +605,32 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
+          <t>「2026년 재난대응 안전한국훈련」국민체험단 모집 공고(공고문)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -642,28 +642,32 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026 고령친화산업 성과교류회 개최 안내</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
+          <t>2026년 스마트 혁신가전 유공자 포상 모집</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -675,7 +679,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -685,7 +689,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
@@ -708,7 +712,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -718,7 +722,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
@@ -729,7 +733,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -741,32 +745,28 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -778,32 +778,32 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
+          <t>2026년 성능인증(EPC) 신규신청 접수 공고(제4차)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -815,32 +815,32 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>K-Startup(창업진흥원)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>구로구 청년창업지원센터 일반 창업교육(하반기: 4회차): 온라인 마케팅 실전 가이드</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>K-Startup(창업진흥원)</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>마케팅</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -852,32 +852,32 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -889,32 +889,32 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -926,32 +926,28 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -963,32 +959,28 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1000,32 +992,28 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1037,32 +1025,32 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1074,32 +1062,32 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1111,32 +1099,32 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
+          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1148,17 +1136,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1168,12 +1156,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1185,32 +1173,32 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>한국산업기술진흥원(KIAT)</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>표창</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1222,32 +1210,32 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1259,7 +1247,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1269,22 +1257,22 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
+          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1296,32 +1284,32 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>전남정보문화산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
+          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1333,32 +1321,32 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
+          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1370,32 +1358,32 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
+          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1407,32 +1395,32 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1444,17 +1432,17 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1464,12 +1452,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1486,27 +1474,27 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>한국산업기술진흥원(KIAT)</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>표창</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1518,32 +1506,32 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>한국사회적기업진흥원</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1555,32 +1543,32 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1592,32 +1580,32 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>전남정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1629,23 +1617,27 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr"/>
+          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1662,28 +1654,32 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr"/>
+          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1695,32 +1691,32 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1732,32 +1728,32 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1769,32 +1765,32 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1806,22 +1802,22 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>한국사회적기업진흥원</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
+          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -1831,7 +1827,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>수출, 스마트</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -1843,7 +1839,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -1853,22 +1849,22 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -1880,17 +1876,17 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1900,12 +1896,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -1917,24 +1913,20 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -1942,7 +1934,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -1954,32 +1946,28 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -1996,27 +1984,27 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
+          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2033,27 +2021,27 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
+          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -2070,27 +2058,27 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -2107,27 +2095,27 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>마케팅, 홍보</t>
+          <t>수출, 스마트</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -2144,27 +2132,27 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -2186,17 +2174,17 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2218,27 +2206,27 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -2260,22 +2248,22 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -2292,27 +2280,27 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, AX</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -2329,27 +2317,27 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -2366,27 +2354,27 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -2403,27 +2391,27 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>마케팅, 홍보</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -2440,27 +2428,27 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>산업통상부</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -2477,23 +2465,27 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>광주정보문화산업진흥원</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr"/>
+          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -2510,23 +2502,27 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr"/>
+          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -2543,33 +2539,321 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
+          <t>중소벤처기업부</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>유공, 포상</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>부산정보산업진흥원</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>에이지테크, AX</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>부산정보산업진흥원</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>에이지테크, 실증</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>광주테크노파크</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>실증</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>광주테크노파크</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Age-Tech</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>산업통상부</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>광주정보문화산업진흥원</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr"/>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
           <t>고령친화산업지원센터</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr"/>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>고령</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr"/>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr"/>
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>고령, 유공, 포상</t>
         </is>
       </c>
-      <c r="G58" s="4" t="inlineStr">
+      <c r="G66" s="4" t="inlineStr">
         <is>
           <t>바로가기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G58"/>
+  <autoFilter ref="A1:G66"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -2628,6 +2912,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId65"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: 발송 이력·누적 기록 갱신 2026-09-25T03:57Z
</commit_message>
<xml_diff>
--- a/공고누적.xlsx
+++ b/공고누적.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공고누적" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -494,32 +494,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>중앙사회서비스원</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -531,32 +531,32 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 원자력안전위원회 최원호 위원장 사퇴 촉구 기자회견</t>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -568,32 +568,32 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 계획 공고</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-11-10</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>「2026년 재난대응 안전한국훈련」국민체험단 모집 공고(공고문)</t>
+          <t>[부산환경운동연합] 원자력안전위원회 최원호 위원장 사퇴 촉구 기자회견</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -647,27 +647,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026년 스마트 혁신가전 유공자 포상 모집</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 계획 공고</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -684,23 +684,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026 고령친화산업 성과교류회 개최 안내</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
+          <t>「2026년 재난대응 안전한국훈련」국민체험단 모집 공고(공고문)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -717,23 +721,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
+          <t>2026년 스마트 혁신가전 유공자 포상 모집</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -755,7 +763,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
@@ -766,7 +774,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -778,32 +786,28 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026년 성능인증(EPC) 신규신청 접수 공고(제4차)</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -815,32 +819,28 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>구로구 청년창업지원센터 일반 창업교육(하반기: 4회차): 온라인 마케팅 실전 가이드</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>마케팅</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -857,27 +857,27 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>2026년 성능인증(EPC) 신규신청 접수 공고(제4차)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -889,32 +889,32 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
+          <t>구로구 청년창업지원센터 일반 창업교육(하반기: 4회차): 온라인 마케팅 실전 가이드</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>마케팅</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -926,28 +926,32 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026 고령친화산업 성과교류회 개최 안내</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -964,23 +968,27 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
+          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1002,7 +1010,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
@@ -1013,7 +1021,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1025,32 +1033,28 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1062,32 +1066,28 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1104,27 +1104,27 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1141,27 +1141,27 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1178,27 +1178,27 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1220,22 +1220,22 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1247,32 +1247,32 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1284,32 +1284,32 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
+          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1341,12 +1341,12 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1358,32 +1358,32 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1395,32 +1395,32 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
+          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1437,27 +1437,27 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
+          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1469,32 +1469,32 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>한국산업기술진흥원(KIAT)</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
+          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>표창</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1506,32 +1506,32 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1548,12 +1548,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국산업기술진흥원(KIAT)</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
+          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1563,12 +1563,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>표창</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1585,12 +1585,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>전남정보문화산업진흥원</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1600,12 +1600,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1622,12 +1622,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
+          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1637,12 +1637,12 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1659,12 +1659,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>전남정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
+          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1674,12 +1674,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1696,27 +1696,27 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1733,17 +1733,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1775,22 +1775,22 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1802,32 +1802,32 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>한국사회적기업진흥원</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -1839,7 +1839,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -1849,22 +1849,22 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -1881,27 +1881,27 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>한국사회적기업진흥원</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -1918,23 +1918,27 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr"/>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -1951,23 +1955,27 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr"/>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -1979,24 +1987,20 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr"/>
       <c r="E43" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -2004,7 +2008,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2016,32 +2020,28 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr"/>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -2058,27 +2058,27 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
+          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -2095,12 +2095,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
+          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2110,12 +2110,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>수출, 스마트</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -2132,27 +2132,27 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -2169,27 +2169,27 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
+          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>수출, 스마트</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -2206,12 +2206,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -2221,12 +2221,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -2243,27 +2243,27 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
+          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -2280,27 +2280,27 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
+          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -2317,12 +2317,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
+          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -2332,12 +2332,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -2354,27 +2354,27 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -2391,27 +2391,27 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>마케팅, 홍보</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -2428,27 +2428,27 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -2465,27 +2465,27 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>마케팅, 홍보</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -2502,27 +2502,27 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -2539,12 +2539,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -2554,12 +2554,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -2576,12 +2576,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2591,12 +2591,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, AX</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -2613,12 +2613,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -2628,12 +2628,12 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -2650,12 +2650,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2665,12 +2665,12 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>에이지테크, AX</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -2687,12 +2687,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>에이지테크, 실증</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -2724,27 +2724,27 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>산업통상부</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -2761,23 +2761,27 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>광주정보문화산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr"/>
+          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -2794,15 +2798,19 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>산업통상부</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr"/>
+          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -2810,7 +2818,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -2827,33 +2835,99 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>광주정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr"/>
       <c r="E66" s="2" t="inlineStr">
         <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr"/>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
           <t>확인필요</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>고령</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr"/>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>고령, 유공, 포상</t>
         </is>
       </c>
-      <c r="G66" s="4" t="inlineStr">
+      <c r="G68" s="4" t="inlineStr">
         <is>
           <t>바로가기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G66"/>
+  <autoFilter ref="A1:G68"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -2920,6 +2994,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId67"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: 발송 이력·누적 기록 갱신 2026-09-28T04:14Z
</commit_message>
<xml_diff>
--- a/공고누적.xlsx
+++ b/공고누적.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공고누적" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -494,32 +494,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+          <t>에이지테크 제품 실증 및 상용화 역량강화 사업 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>에이지테크, 실증</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -531,32 +531,32 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>2026년 경남 해양수산 창업투자지원사업 수출 물류비 지원 수혜기업 모집 공고</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -568,22 +568,22 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 연장 공고</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -605,32 +605,32 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 원자력안전위원회 최원호 위원장 사퇴 촉구 기자회견</t>
+          <t>2027년 생산단계 축산물 스마트 HACCP 현장구축 사업 대상자(도축장·집유장 영업자) 모집 공고</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -642,27 +642,27 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 계획 공고</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-11-10</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -679,32 +679,32 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>「2026년 재난대응 안전한국훈련」국민체험단 모집 공고(공고문)</t>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -716,32 +716,32 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026년 스마트 혁신가전 유공자 포상 모집</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -758,23 +758,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026 고령친화산업 성과교류회 개최 안내</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
+          <t>[부산환경운동연합] 원자력안전위원회 최원호 위원장 사퇴 촉구 기자회견</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -791,23 +795,27 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 계획 공고</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -824,23 +832,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
+          <t>「2026년 재난대응 안전한국훈련」국민체험단 모집 공고(공고문)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -852,32 +864,32 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026년 성능인증(EPC) 신규신청 접수 공고(제4차)</t>
+          <t>2026년 스마트 혁신가전 유공자 포상 모집</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -889,32 +901,28 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>구로구 청년창업지원센터 일반 창업교육(하반기: 4회차): 온라인 마케팅 실전 가이드</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>마케팅</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -926,32 +934,28 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -963,32 +967,28 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1000,28 +1000,32 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2026 고령친화산업 성과교류회 개최 안내</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
+          <t>2026년 성능인증(EPC) 신규신청 접수 공고(제4차)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1033,28 +1037,32 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
+          <t>구로구 청년창업지원센터 일반 창업교육(하반기: 4회차): 온라인 마케팅 실전 가이드</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>마케팅</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1066,28 +1074,32 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1099,32 +1111,32 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1136,32 +1148,28 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1173,32 +1181,28 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1210,32 +1214,28 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1257,12 +1257,12 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1289,27 +1289,27 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1321,32 +1321,32 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
+          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1358,32 +1358,32 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1395,32 +1395,32 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1432,22 +1432,22 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1469,32 +1469,32 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
+          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1506,32 +1506,32 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
+          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1543,32 +1543,32 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>한국산업기술진흥원(KIAT)</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
+          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>표창</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1580,32 +1580,32 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1617,32 +1617,32 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
+          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1654,32 +1654,32 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>전남정보문화산업진흥원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
+          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1696,12 +1696,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국산업기술진흥원(KIAT)</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
+          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1711,12 +1711,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>표창</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1733,12 +1733,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1748,12 +1748,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1770,27 +1770,27 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1807,27 +1807,27 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>전남정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -1844,17 +1844,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -1876,32 +1876,32 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>한국사회적기업진흥원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
+          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -1913,32 +1913,32 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>한국보건산업진흥원</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -1950,32 +1950,32 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>한국보건산업진흥원</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -1987,28 +1987,32 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr"/>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2025,15 +2029,19 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국사회적기업진흥원</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr"/>
+          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -2041,7 +2049,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -2053,32 +2061,32 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -2090,32 +2098,32 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -2127,32 +2135,28 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -2164,24 +2168,20 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr"/>
       <c r="E48" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>수출, 스마트</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -2206,27 +2206,27 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -2243,27 +2243,27 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
+          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -2280,27 +2280,27 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
+          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -2317,27 +2317,27 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
+          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>수출, 스마트</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -2354,27 +2354,27 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -2391,27 +2391,27 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
+          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -2428,27 +2428,27 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -2465,27 +2465,27 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>마케팅, 홍보</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -2502,27 +2502,27 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -2539,27 +2539,27 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -2581,22 +2581,22 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -2613,27 +2613,27 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>마케팅, 홍보</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -2650,27 +2650,27 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, AX</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -2687,12 +2687,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -2702,12 +2702,12 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -2724,12 +2724,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -2739,12 +2739,12 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -2761,12 +2761,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2776,12 +2776,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -2798,27 +2798,27 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>산업통상부</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>에이지테크, AX</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -2835,23 +2835,27 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>광주정보문화산업진흥원</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr"/>
+          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>에이지테크, 실증</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -2868,23 +2872,27 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr"/>
+          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
@@ -2901,33 +2909,173 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
+          <t>광주테크노파크</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Age-Tech</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>산업통상부</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>광주정보문화산업진흥원</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr"/>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
           <t>고령친화산업지원센터</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr">
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr"/>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>고령</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
         <is>
           <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr"/>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr"/>
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>고령, 유공, 포상</t>
         </is>
       </c>
-      <c r="G68" s="4" t="inlineStr">
+      <c r="G72" s="4" t="inlineStr">
         <is>
           <t>바로가기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G68"/>
+  <autoFilter ref="A1:G72"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -2996,6 +3144,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId71"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: 발송 이력·누적 기록 갱신 2026-09-30T04:50Z
</commit_message>
<xml_diff>
--- a/공고누적.xlsx
+++ b/공고누적.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공고누적" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -494,32 +494,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>에이지테크 제품 실증 및 상용화 역량강화 사업 수혜기업 모집공고</t>
+          <t>2027년 지자체 연계 의료기기 신규 지원사업 참여 수요조사(~10/23)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -531,32 +531,32 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2026년 경남 해양수산 창업투자지원사업 수출 물류비 지원 수혜기업 모집 공고</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -568,32 +568,32 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 연장 공고</t>
+          <t>2027년 지자체 연계 의료기기 신규 지원사업 참여 수요조사(~10/23)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -605,22 +605,22 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2027년 생산단계 축산물 스마트 HACCP 현장구축 사업 대상자(도축장·집유장 영업자) 모집 공고</t>
+          <t>2026년 사회서비스 기업 온라인 상담 서비스 운영 안내</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -642,32 +642,32 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+          <t>2026년 상반기 기관생명윤리위원회 평가 인증(신규) 결과 공고</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -679,32 +679,32 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>2026년 스마트공장 사전사후 컨설팅사업 지원기업 모집공고</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -716,32 +716,32 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>광주경제진흥상생일자리재단</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>2026년 K-브랜드 정부인증제도 참여기업 모집 공고…</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -753,32 +753,32 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 원자력안전위원회 최원호 위원장 사퇴 촉구 기자회견</t>
+          <t>AI 올라운더(기획,개발,마케팅) 창업가육성과정 8기 모집</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>마케팅</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -790,27 +790,27 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 계획 공고</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-11-10</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -827,32 +827,32 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>「2026년 재난대응 안전한국훈련」국민체험단 모집 공고(공고문)</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -864,32 +864,32 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026년 스마트 혁신가전 유공자 포상 모집</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -901,28 +901,32 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>K-Startup(창업진흥원)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>2026 「Go to Market」동남권 창업기업 온라인 판로개척 교육 참가자 모집</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>고령친화산업지원센터</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>2026 고령친화산업 성과교류회 개최 안내</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -934,7 +938,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -944,18 +948,18 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+          <t>[공고] 'Age-Tech 종합지원센터 지원사업' 참여기관 모집 공고(~ 3.30(월) 17:00까지)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2027-03-30</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -967,28 +971,32 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 연장 공고</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1000,32 +1008,32 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2026년 성능인증(EPC) 신규신청 접수 공고(제4차)</t>
+          <t>2027년 생산단계 축산물 스마트 HACCP 현장구축 사업 대상자(도축장·집유장 영업자) 모집 공고</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1037,32 +1045,32 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>구로구 청년창업지원센터 일반 창업교육(하반기: 4회차): 온라인 마케팅 실전 가이드</t>
+          <t>에이지테크 제품 실증 및 상용화 역량강화 사업 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>마케팅</t>
+          <t>에이지테크, 실증</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1074,22 +1082,22 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>2026년 경남 해양수산 창업투자지원사업 수출 물류비 지원 수혜기업 모집 공고</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1099,7 +1107,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1111,32 +1119,32 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1148,28 +1156,32 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>2026 고령친화산업 성과교류회 개최 안내</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1181,28 +1193,32 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1214,28 +1230,32 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
+          <t>[부산환경운동연합] 원자력안전위원회 최원호 위원장 사퇴 촉구 기자회견</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1247,32 +1267,32 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 계획 공고</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1284,32 +1304,32 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
+          <t>「2026년 재난대응 안전한국훈련」국민체험단 모집 공고(공고문)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1321,7 +1341,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1331,22 +1351,22 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
+          <t>2026년 스마트 혁신가전 유공자 포상 모집</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1358,32 +1378,28 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1395,32 +1411,28 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1432,32 +1444,28 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1469,7 +1477,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1479,22 +1487,22 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
+          <t>2026년 성능인증(EPC) 신규신청 접수 공고(제4차)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1506,22 +1514,22 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
+          <t>구로구 청년창업지원센터 일반 창업교육(하반기: 4회차): 온라인 마케팅 실전 가이드</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1531,7 +1539,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>마케팅</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1543,32 +1551,32 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1580,32 +1588,32 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1617,32 +1625,28 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1654,32 +1658,28 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1691,32 +1691,28 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>한국산업기술진흥원(KIAT)</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>표창</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1728,32 +1724,32 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1765,32 +1761,32 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
+          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1802,32 +1798,32 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>K-Startup(창업진흥원)</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>전남정보문화산업진흥원</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -1839,32 +1835,32 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -1876,22 +1872,22 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -1901,7 +1897,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -1913,7 +1909,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -1923,22 +1919,22 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -1950,32 +1946,32 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -1987,32 +1983,32 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2024,32 +2020,32 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>한국사회적기업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
+          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -2061,32 +2057,32 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -2098,32 +2094,32 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -2135,28 +2131,32 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>K-Startup(창업진흥원)</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>고령친화산업지원센터</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -2168,28 +2168,32 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국산업기술진흥원(KIAT)</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr"/>
+          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>표창</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -2201,32 +2205,32 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -2238,32 +2242,32 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
+          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -2275,32 +2279,32 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>전남정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
+          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -2312,32 +2316,32 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
+          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>수출, 스마트</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -2349,32 +2353,32 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -2386,32 +2390,32 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -2423,32 +2427,32 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -2460,32 +2464,32 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -2497,32 +2501,32 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국사회적기업진흥원</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
+          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -2534,22 +2538,22 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2559,7 +2563,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -2571,32 +2575,32 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -2608,32 +2612,28 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr"/>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>마케팅, 홍보</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -2645,32 +2645,28 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr"/>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -2687,27 +2683,27 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -2724,27 +2720,27 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -2761,27 +2757,27 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -2798,27 +2794,27 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, AX</t>
+          <t>수출, 스마트</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -2835,27 +2831,27 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -2872,27 +2868,27 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
@@ -2909,27 +2905,27 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
@@ -2946,27 +2942,27 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>산업통상부</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -2983,23 +2979,27 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>광주정보문화산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr"/>
+          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
@@ -3016,23 +3016,27 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr"/>
+          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
@@ -3049,33 +3053,506 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
+          <t>중소벤처기업부</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>유공, 포상, 스마트</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>경남테크노파크</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>마케팅, 홍보</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>보건복지부</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>유공, 포상</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>중앙사회서비스원</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>사회서비스</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>중소벤처기업부</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>중소벤처기업부</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>유공, 포상</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>부산정보산업진흥원</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>에이지테크, AX</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>부산정보산업진흥원</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>에이지테크, 실증</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>광주테크노파크</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>실증</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>광주테크노파크</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Age-Tech</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>산업통상부</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>광주정보문화산업진흥원</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr"/>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
           <t>고령친화산업지원센터</t>
         </is>
       </c>
-      <c r="C72" s="3" t="inlineStr">
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr"/>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>고령</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
         <is>
           <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr"/>
-      <c r="E72" s="2" t="inlineStr">
+      <c r="D85" s="2" t="inlineStr"/>
+      <c r="E85" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr">
+      <c r="F85" s="2" t="inlineStr">
         <is>
           <t>고령, 유공, 포상</t>
         </is>
       </c>
-      <c r="G72" s="4" t="inlineStr">
+      <c r="G85" s="4" t="inlineStr">
         <is>
           <t>바로가기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G72"/>
+  <autoFilter ref="A1:G85"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -3148,6 +3625,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId84"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: 발송 이력·누적 기록 갱신 2026-09-30T14:32Z
</commit_message>
<xml_diff>
--- a/공고누적.xlsx
+++ b/공고누적.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공고누적" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -504,17 +504,17 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2027년 지자체 연계 의료기기 신규 지원사업 참여 수요조사(~10/23)</t>
+          <t>2027 WHX Dubai 및 WHX Tech 연계 한국의료기기 통합전시관 및 세미나 발표 기업 모집공고 (10.16(금), 18:00까지)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -541,22 +541,22 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+          <t>2027년 지자체 연계 의료기기 신규 지원사업 참여 수요조사(~10/23)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -568,7 +568,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -605,32 +605,32 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 기업 온라인 상담 서비스 운영 안내</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -642,32 +642,32 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026년 상반기 기관생명윤리위원회 평가 인증(신규) 결과 공고</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -684,27 +684,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026년 스마트공장 사전사후 컨설팅사업 지원기업 모집공고</t>
+          <t>2027년 지자체 연계 의료기기 신규 지원사업 참여 수요조사(~10/23)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -721,17 +721,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>광주경제진흥상생일자리재단</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026년 K-브랜드 정부인증제도 참여기업 모집 공고…</t>
+          <t>2026년 사회서비스 기업 온라인 상담 서비스 운영 안내</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -758,27 +758,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>AI 올라운더(기획,개발,마케팅) 창업가육성과정 8기 모집</t>
+          <t>2026년 상반기 기관생명윤리위원회 평가 인증(신규) 결과 공고</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>마케팅</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -795,27 +795,27 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+          <t>2026년 스마트공장 사전사후 컨설팅사업 지원기업 모집공고</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -832,27 +832,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>광주경제진흥상생일자리재단</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+          <t>2026년 K-브랜드 정부인증제도 참여기업 모집 공고…</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -869,27 +869,27 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+          <t>AI 올라운더(기획,개발,마케팅) 창업가육성과정 8기 모집</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>마케팅</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -906,27 +906,27 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026 「Go to Market」동남권 창업기업 온라인 판로개척 교육 참가자 모집</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -943,23 +943,27 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>[공고] 'Age-Tech 종합지원센터 지원사업' 참여기관 모집 공고(~ 3.30(월) 17:00까지)</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2027-03-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -971,32 +975,32 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 연장 공고</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1008,32 +1012,32 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2027년 생산단계 축산물 스마트 HACCP 현장구축 사업 대상자(도축장·집유장 영업자) 모집 공고</t>
+          <t>2026 「Go to Market」동남권 창업기업 온라인 판로개척 교육 참가자 모집</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1045,32 +1049,28 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>에이지테크 제품 실증 및 상용화 역량강화 사업 수혜기업 모집공고</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>[공고] 'Age-Tech 종합지원센터 지원사업' 참여기관 모집 공고(~ 3.30(월) 17:00까지)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2027-03-30</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1087,12 +1087,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026년 경남 해양수산 창업투자지원사업 수출 물류비 지원 수혜기업 모집 공고</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 연장 공고</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1119,32 +1119,32 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+          <t>2027년 생산단계 축산물 스마트 HACCP 현장구축 사업 대상자(도축장·집유장 영업자) 모집 공고</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1156,32 +1156,32 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>에이지테크 제품 실증 및 상용화 역량강화 사업 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>에이지테크, 실증</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1193,22 +1193,22 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>2026년 경남 해양수산 창업투자지원사업 수출 물류비 지원 수혜기업 모집 공고</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1230,32 +1230,32 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 원자력안전위원회 최원호 위원장 사퇴 촉구 기자회견</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1267,32 +1267,32 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 계획 공고</t>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>2026-11-10</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1304,32 +1304,32 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>「2026년 재난대응 안전한국훈련」국민체험단 모집 공고(공고문)</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1346,27 +1346,27 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>2026년 스마트 혁신가전 유공자 포상 모집</t>
+          <t>[부산환경운동연합] 원자력안전위원회 최원호 위원장 사퇴 촉구 기자회견</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1383,23 +1383,27 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>2026 고령친화산업 성과교류회 개최 안내</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 계획 공고</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1416,23 +1420,27 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
+          <t>「2026년 재난대응 안전한국훈련」국민체험단 모집 공고(공고문)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1449,23 +1457,27 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr"/>
+          <t>2026년 스마트 혁신가전 유공자 포상 모집</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1477,32 +1489,28 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>2026년 성능인증(EPC) 신규신청 접수 공고(제4차)</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1514,32 +1522,28 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>구로구 청년창업지원센터 일반 창업교육(하반기: 4회차): 온라인 마케팅 실전 가이드</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>마케팅</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1551,32 +1555,28 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1588,27 +1588,27 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
+          <t>2026년 성능인증(EPC) 신규신청 접수 공고(제4차)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1625,28 +1625,32 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>2026 고령친화산업 성과교류회 개최 안내</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr"/>
+          <t>구로구 청년창업지원센터 일반 창업교육(하반기: 4회차): 온라인 마케팅 실전 가이드</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>마케팅</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1658,28 +1662,32 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr"/>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1696,23 +1704,27 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr"/>
+          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1724,32 +1736,28 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1761,32 +1769,28 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1798,32 +1802,28 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -1845,22 +1845,22 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -1877,27 +1877,27 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -1914,27 +1914,27 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -1946,32 +1946,32 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -1983,32 +1983,32 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2020,32 +2020,32 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -2057,22 +2057,22 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -2094,32 +2094,32 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
+          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -2131,32 +2131,32 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
+          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -2168,32 +2168,32 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>한국산업기술진흥원(KIAT)</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
+          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>표창</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -2205,32 +2205,32 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -2242,32 +2242,32 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
+          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -2284,12 +2284,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>전남정보문화산업진흥원</t>
+          <t>한국산업기술진흥원(KIAT)</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
+          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2299,12 +2299,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>표창</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -2321,12 +2321,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -2336,12 +2336,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -2358,12 +2358,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
+          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2373,12 +2373,12 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -2395,27 +2395,27 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>전남정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -2432,27 +2432,27 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -2469,27 +2469,27 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -2501,32 +2501,32 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>한국사회적기업진흥원</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -2538,7 +2538,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2575,7 +2575,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2617,15 +2617,19 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국사회적기업진흥원</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr"/>
+          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -2633,7 +2637,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -2650,23 +2654,27 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr"/>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -2678,32 +2686,32 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -2715,32 +2723,28 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr"/>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -2752,32 +2756,28 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr"/>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -2794,17 +2794,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
+          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>수출, 스마트</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -2831,27 +2831,27 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -2868,27 +2868,27 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
+          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
@@ -2910,12 +2910,12 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
+          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>수출, 스마트</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
@@ -2942,27 +2942,27 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -2979,27 +2979,27 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
+          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
@@ -3016,27 +3016,27 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
+          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
@@ -3058,22 +3058,22 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
@@ -3090,27 +3090,27 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>마케팅, 홍보</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
@@ -3127,27 +3127,27 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
@@ -3164,27 +3164,27 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
@@ -3201,27 +3201,27 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>마케팅, 홍보</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
@@ -3238,22 +3238,22 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -3275,12 +3275,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -3290,12 +3290,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, AX</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
@@ -3312,12 +3312,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -3327,12 +3327,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
@@ -3349,12 +3349,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -3364,12 +3364,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
@@ -3386,12 +3386,12 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>에이지테크, AX</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
@@ -3423,27 +3423,27 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>산업통상부</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>에이지테크, 실증</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
@@ -3460,23 +3460,27 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>광주정보문화산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr"/>
+          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr">
@@ -3493,23 +3497,27 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr"/>
+          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr">
@@ -3526,33 +3534,136 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
+          <t>산업통상부</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>광주정보문화산업진흥원</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr"/>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
           <t>고령친화산업지원센터</t>
         </is>
       </c>
-      <c r="C85" s="3" t="inlineStr">
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr"/>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>고령</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
         <is>
           <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
         </is>
       </c>
-      <c r="D85" s="2" t="inlineStr"/>
-      <c r="E85" s="2" t="inlineStr">
+      <c r="D88" s="2" t="inlineStr"/>
+      <c r="E88" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr">
+      <c r="F88" s="2" t="inlineStr">
         <is>
           <t>고령, 유공, 포상</t>
         </is>
       </c>
-      <c r="G85" s="4" t="inlineStr">
+      <c r="G88" s="4" t="inlineStr">
         <is>
           <t>바로가기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G85"/>
+  <autoFilter ref="A1:G88"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -3638,6 +3749,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId87"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: 발송 이력·누적 기록 갱신 2026-10-02T04:35Z
</commit_message>
<xml_diff>
--- a/공고누적.xlsx
+++ b/공고누적.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공고누적" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공고누적'!$A$1:$G$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -494,32 +494,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>정보통신산업진흥원(NIPA)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2027 WHX Dubai 및 WHX Tech 연계 한국의료기기 통합전시관 및 세미나 발표 기업 모집공고 (10.16(금), 18:00까지)</t>
+          <t>2026년도 고용노동부(안전보건공단) 연계 스마트 안전장비지원 품목 등록 시행계획 공고 2차</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>안전, 스마트</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -531,27 +531,27 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>2027 WHX Dubai 및 WHX Tech 연계 한국의료기기 통합전시관 및 세미나 발표 기업 모집공고 (10.16(금), 18:00까지)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>한국보건산업진흥원</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>2027년 지자체 연계 의료기기 신규 지원사업 참여 수요조사(~10/23)</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -568,7 +568,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -605,7 +605,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -652,22 +652,22 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+          <t>2027 WHX Dubai 및 WHX Tech 연계 한국의료기기 통합전시관 및 세미나 발표 기업 모집공고 (10.16(금), 18:00까지)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -679,7 +679,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -716,32 +716,32 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>2027년 지자체 연계 의료기기 신규 지원사업 참여 수요조사(~10/23)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>중앙사회서비스원</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>2026년 사회서비스 기업 온라인 상담 서비스 운영 안내</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -753,32 +753,32 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026년 상반기 기관생명윤리위원회 평가 인증(신규) 결과 공고</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -790,32 +790,32 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026년 스마트공장 사전사후 컨설팅사업 지원기업 모집공고</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -832,27 +832,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>광주경제진흥상생일자리재단</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026년 K-브랜드 정부인증제도 참여기업 모집 공고…</t>
+          <t>2027년 지자체 연계 의료기기 신규 지원사업 참여 수요조사(~10/23)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -869,27 +869,27 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>AI 올라운더(기획,개발,마케팅) 창업가육성과정 8기 모집</t>
+          <t>2026년 사회서비스 기업 온라인 상담 서비스 운영 안내</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>마케팅</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -906,27 +906,27 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+          <t>2026년 상반기 기관생명윤리위원회 평가 인증(신규) 결과 공고</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -943,27 +943,27 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+          <t>2026년 스마트공장 사전사후 컨설팅사업 지원기업 모집공고</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -980,27 +980,27 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>광주경제진흥상생일자리재단</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+          <t>2026년 K-브랜드 정부인증제도 참여기업 모집 공고…</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1022,22 +1022,22 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2026 「Go to Market」동남권 창업기업 온라인 판로개척 교육 참가자 모집</t>
+          <t>AI 올라운더(기획,개발,마케팅) 창업가육성과정 8기 모집</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>마케팅</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1054,23 +1054,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>[공고] 'Age-Tech 종합지원센터 지원사업' 참여기관 모집 공고(~ 3.30(월) 17:00까지)</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2027-03-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1082,32 +1086,32 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 연장 공고</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1119,32 +1123,32 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2027년 생산단계 축산물 스마트 HACCP 현장구축 사업 대상자(도축장·집유장 영업자) 모집 공고</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1156,32 +1160,32 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>에이지테크 제품 실증 및 상용화 역량강화 사업 수혜기업 모집공고</t>
+          <t>2026 「Go to Market」동남권 창업기업 온라인 판로개척 교육 참가자 모집</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1193,32 +1197,28 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>2026년 경남 해양수산 창업투자지원사업 수출 물류비 지원 수혜기업 모집 공고</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>[공고] 'Age-Tech 종합지원센터 지원사업' 참여기관 모집 공고(~ 3.30(월) 17:00까지)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2027-03-30</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1230,32 +1230,32 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 연장 공고</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>헬스케어, 유공, 포상</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1267,32 +1267,32 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>2027년 생산단계 축산물 스마트 HACCP 현장구축 사업 대상자(도축장·집유장 영업자) 모집 공고</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1304,32 +1304,32 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>에이지테크 제품 실증 및 상용화 역량강화 사업 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>에이지테크, 실증</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1341,32 +1341,32 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 원자력안전위원회 최원호 위원장 사퇴 촉구 기자회견</t>
+          <t>2026년 경남 해양수산 창업투자지원사업 수출 물류비 지원 수혜기업 모집 공고</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1378,27 +1378,27 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 계획 공고</t>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 추천 후보자 접수(~10.30(금)24:00까지</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>2026-11-10</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1415,32 +1415,32 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>「2026년 재난대응 안전한국훈련」국민체험단 모집 공고(공고문)</t>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1452,32 +1452,32 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>2026년 스마트 혁신가전 유공자 포상 모집</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1494,23 +1494,27 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>2026 고령친화산업 성과교류회 개최 안내</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr"/>
+          <t>[부산환경운동연합] 원자력안전위원회 최원호 위원장 사퇴 촉구 기자회견</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1527,23 +1531,27 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
+          <t>2027 메디컬 코리아 글로벌 헬스케어 유공 포상 계획 공고</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>헬스케어, 유공, 포상</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1560,23 +1568,27 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr"/>
+          <t>「2026년 재난대응 안전한국훈련」국민체험단 모집 공고(공고문)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1588,32 +1600,32 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>2026년 성능인증(EPC) 신규신청 접수 공고(제4차)</t>
+          <t>2026년 스마트 혁신가전 유공자 포상 모집</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1625,32 +1637,28 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>구로구 청년창업지원센터 일반 창업교육(하반기: 4회차): 온라인 마케팅 실전 가이드</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>마케팅</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1662,32 +1670,28 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1699,32 +1703,28 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1736,28 +1736,32 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>2026 고령친화산업 성과교류회 개최 안내</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr"/>
+          <t>2026년 성능인증(EPC) 신규신청 접수 공고(제4차)</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1769,28 +1773,32 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr"/>
+          <t>구로구 청년창업지원센터 일반 창업교육(하반기: 4회차): 온라인 마케팅 실전 가이드</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>마케팅</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1802,28 +1810,32 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr"/>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -1835,32 +1847,32 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>「2026 ‘Made in BUSA 신발’ 정품인증 레이블 지원」 수요기업 모집(2차) 공고</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -1872,32 +1884,28 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+          <t>2026 고령친화산업 성과교류회 개최 안내</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -1909,32 +1917,28 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -1946,32 +1950,28 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -1993,12 +1993,12 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -2025,27 +2025,27 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년 반도체 첨단패키징 실증센터 구축사업 수혜기업 3차 모집공고</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -2057,32 +2057,32 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
+          <t>[부산대학교병원]「의료·헬스케어 스타트업 인큐베이터 사업」국내전시회(공동관) 참가지원 모집 공고</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -2094,32 +2094,32 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -2131,32 +2131,32 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -2168,22 +2168,22 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -2205,32 +2205,32 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
+          <t>2026년 온라인수출 중소기업 물류 지원사업 참여기업 모집 공고(연장)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -2242,32 +2242,32 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
+          <t>2027년 수출컨소시엄 사업 주관단체 및 과제 모집 공고</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -2279,32 +2279,32 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>한국산업기술진흥원(KIAT)</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
+          <t>2027년 스마트공장 구축지원사업 주관기관 모집 공고</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>표창</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -2316,32 +2316,32 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
+          <t>2026-727호] 2026년도 혁신형 제약기업 및 제약산업 발전 유공자 포상 공고</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -2353,32 +2353,32 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
+          <t>"2026년 앵커(ANCHOR) R&amp;D기반 혁신 실증스튜디오 운영 사업" 실증프로세스 및 AI적용 성공사례 벤치마킹 교육 위탁수행기관(업) 모집 공고</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -2390,32 +2390,32 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>전남정보문화산업진흥원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
+          <t>제3회 AI 및 기술기반 창업 트렌드 세미나 참가자 모집 (AI 비즈니스 실전 전략 : 멀티모달·에이전트 AX·AI 거버넌스)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -2432,12 +2432,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국산업기술진흥원(KIAT)</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
+          <t>2026년도 제4회 중견기업 혁신대상 장관표창 계획 공고</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -2447,12 +2447,12 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>표창</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -2469,12 +2469,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
+          <t>2026년 사회서비스 종사자 심리지원사업 집단프로그램 참여기관 모집(~10/2)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -2484,12 +2484,12 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -2506,27 +2506,27 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+          <t>「2026년 상생결제 확산 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>의료기기</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -2543,27 +2543,27 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>전남정보문화산업진흥원</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+          <t>아태 AI 특화지구(AHAP) 조성사업-AX 실증 지원 사전 수요조사(9/14~9/16)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>AX, 실증</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -2580,17 +2580,17 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>2026년도 부산광역시 고령친화산업 육성 지원사업 지역기업 역량강화 교육생 모집 공고(연장~9.30.) 연장</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -2600,7 +2600,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -2612,32 +2612,32 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>한국사회적기업진흥원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
+          <t>2026-358 2026 태국 방산수출사절단 참가지원사업(2차) 참가기업 공고문</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -2649,32 +2649,32 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>2026년 글로벌 규제 대응 비용 지원(의료기기) 사업 수행기업 모집 3차 공고(9월 28일(월) 18시까지)</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>한국보건산업진흥원</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>홍보</t>
+          <t>의료기기</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -2686,32 +2686,32 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>한국보건산업진흥원</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>한국보건산업진흥원</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -2723,28 +2723,32 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr"/>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -2761,15 +2765,19 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>한국사회적기업진흥원</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr"/>
+          <t>[고용노동부 공고] 2026년 제3차 사회적기업 인증 공고</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -2777,7 +2785,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>고령, 유공, 포상</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -2789,32 +2797,32 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>부산시민운동지원센터</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
+          <t>「2026 한-카자흐스탄 보건의료 해외진출 홍보 및 공공조달 협력 세미나」 참가기관 모집 공고(~9.18(금) 18:00)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>안전</t>
+          <t>홍보</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -2826,32 +2834,32 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>인증</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -2863,32 +2871,28 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr"/>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>고령</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
@@ -2900,24 +2904,20 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>고령친화산업지원센터</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
+          <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr"/>
       <c r="E68" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>수출, 스마트</t>
+          <t>고령, 유공, 포상</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
@@ -2942,27 +2942,27 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>한국보건산업진흥원</t>
+          <t>부산시민운동지원센터</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
+          <t>[부산환경운동연합] 고리3·4호기 사고관리계획서 원자력안전위원회 일괄 안건 상정에 따른 긴급 기자회견</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>디지털헬스, 헬스케어</t>
+          <t>안전</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -2979,27 +2979,27 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
+          <t>2026년 수리조선 기업인증 지원사업 추가모집 공고 재공고</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>인증</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
@@ -3016,27 +3016,27 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>농림축산식품부</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
+          <t>「부산 AX클리닉」 지원기업 2차 모집공고(~ 9. 18.(금) 16:00)</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
@@ -3053,27 +3053,27 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
+          <t>'27년 스마트 수출전문단지 구축 사업 공모</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>스마트</t>
+          <t>수출, 스마트</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
@@ -3090,27 +3090,27 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>부산테크노파크</t>
+          <t>한국보건산업진흥원</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
+          <t>[공고] 「HLTH USA 2026」 디지털헬스케어 한국관 참가기관 모집 공고(~9.30.(수)) 15시까지</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>디지털헬스, 헬스케어</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
@@ -3127,27 +3127,27 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>K-Startup(창업진흥원)</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
+          <t>「2026년 제2차 사회서비스 정책포럼」 개최 안내</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>판로</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
@@ -3164,27 +3164,27 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>농림축산식품부</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
+          <t>스마트팜 다부처 패키지 혁신기술개발 후속사업 기획 및 스마트팜 고도화를 위한 현장 의견 조사</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상, 스마트</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
@@ -3201,27 +3201,27 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
+          <t>2026년 중소기업 스마트서비스 지원사업 참여기업 모집 공고(A/S지원)</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>마케팅, 홍보</t>
+          <t>스마트</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
@@ -3238,27 +3238,27 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>보건복지부</t>
+          <t>부산테크노파크</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
+          <t>Age-Tech 종합지원센터 운영 사업 TRL기반 기술성장 맞춤 지원 공고</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>Age-Tech</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr">
@@ -3275,27 +3275,27 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>중앙사회서비스원</t>
+          <t>K-Startup(창업진흥원)</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
+          <t>[서초창업스테이션] 9월 창업 교육 - 스타트업을 위한 온라인 판로개척</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>사회서비스</t>
+          <t>판로</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
@@ -3317,22 +3317,22 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
+          <t>「2026년 스마트제조혁신 유공」 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>유공, 포상, 스마트</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
@@ -3349,27 +3349,27 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>중소벤처기업부</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
+          <t>경상남도 제조 스타트업 홍보·마케팅 지원 프로그램 수혜기업 모집공고</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>유공, 포상</t>
+          <t>마케팅, 홍보</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
@@ -3386,27 +3386,27 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>보건복지부</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
+          <t>2026년 드림스타트 사업 유공자 포상 추천 공고</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, AX</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
@@ -3423,12 +3423,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>부산정보산업진흥원</t>
+          <t>중앙사회서비스원</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+          <t>2026년 사회서비스 종사자 심리상담 지원사업 3기 참여자 모집(~9/30)</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -3438,12 +3438,12 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>에이지테크, 실증</t>
+          <t>사회서비스</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
@@ -3460,12 +3460,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+          <t>『중소기업 AX 우수사례 공모전』참가기업 모집 공고</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -3475,12 +3475,12 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr">
@@ -3497,12 +3497,12 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>광주테크노파크</t>
+          <t>중소벤처기업부</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+          <t>「지역 중소기업 AI 활용·확산 유공 포상」 후보자 모집 공고</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -3512,12 +3512,12 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Age-Tech</t>
+          <t>유공, 포상</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr">
@@ -3534,27 +3534,27 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>산업통상부</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+          <t>2026년 AX 에이지테크 시장확산 지원사업 모집 공고</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>에이지테크, AX</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr">
@@ -3571,23 +3571,27 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>광주정보문화산업진흥원</t>
+          <t>부산정보산업진흥원</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr"/>
+          <t>2026 해양문화도시 기반의 에이지테크 실증거점 조성 사업 「CES 2027 통합 부산관」 참가기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>AX, 실증</t>
+          <t>에이지테크, 실증</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr">
@@ -3604,23 +3608,27 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>고령친화산업지원센터</t>
+          <t>광주테크노파크</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
-        </is>
-      </c>
-      <c r="D87" s="2" t="inlineStr"/>
+          <t>「2026년도 연구개발특구진흥재단 광주특구본부」 지역혁신 실증 프로젝트 기획 실증의제 수요조사 공고(2차)</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>고령</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="G87" s="4" t="inlineStr">
@@ -3637,33 +3645,173 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
+          <t>광주테크노파크</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Age-Tech 제품 사용성평가 참여자 모집 공고</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Age-Tech</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>산업통상부</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>2026년도 AX실증밸리조성(R&amp;D) 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>광주정보문화산업진흥원</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>아태 AI 특화지구(AHAP) 조성 사업 AX 실증 사전 수요조사</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr"/>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>AX, 실증</t>
+        </is>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
           <t>고령친화산업지원센터</t>
         </is>
       </c>
-      <c r="C88" s="3" t="inlineStr">
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>[공고] 2026년 1차 고령친화우수제품 지정 공고</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr"/>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>고령</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>바로가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>고령친화산업지원센터</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
         <is>
           <t>[공고] 2026년 고령친화산업 육성 유공자 정부 포상 추천계획 공고</t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr"/>
-      <c r="E88" s="2" t="inlineStr">
+      <c r="D92" s="2" t="inlineStr"/>
+      <c r="E92" s="2" t="inlineStr">
         <is>
           <t>확인필요</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr">
+      <c r="F92" s="2" t="inlineStr">
         <is>
           <t>고령, 유공, 포상</t>
         </is>
       </c>
-      <c r="G88" s="4" t="inlineStr">
+      <c r="G92" s="4" t="inlineStr">
         <is>
           <t>바로가기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G88"/>
+  <autoFilter ref="A1:G92"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -3752,6 +3900,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId91"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>